<commit_message>
immobilier : bascule sur DVF (prix reels) + Carte des loyers 2025
</commit_message>
<xml_diff>
--- a/data/output/grille_ponderation_lille.xlsx
+++ b/data/output/grille_ponderation_lille.xlsx
@@ -917,7 +917,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>cadre_urbain_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>SeLoger/MeilleursAgents avril 2026 ; winsor DEUX queues : les prix planchers (marche en detresse) ne doivent pas scorer 20/20</t>
+          <t>DVF transactions reelles 2023-2025 (mediane communale) ; winsor DEUX queues : les prix planchers (marche en detresse) ne scorent pas 20/20</t>
         </is>
       </c>
     </row>
@@ -960,17 +960,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>prix_appart_m2</t>
+          <t>loyers_maison_m2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Prix des appartements au m2</t>
+          <t>Loyers des maisons au m2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>cadre_urbain_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -991,7 +991,11 @@
           <t>mediane</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Carte des loyers 2025 (indicateur d'annonce predit, CGDD/ANIL)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1009,17 +1013,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>loyers_maison_m2</t>
+          <t>loyers_appart_m2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Loyers des maisons au m2</t>
+          <t>Loyers des appartements au m2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>cadre_urbain_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1040,7 +1044,11 @@
           <t>mediane</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Carte des loyers 2025 ; pertinent surtout pour les communes MEL (locatif)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2641,7 +2649,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
scoring v2 : 10 themes + dynamique + cout_logement + log + bonus/malus + tranches + robustesse
</commit_message>
<xml_diff>
--- a/data/output/grille_ponderation_lille.xlsx
+++ b/data/output/grille_ponderation_lille.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteres &amp; ponderation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recap themes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preset defaut" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteres" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus-malus" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recap themes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preset defaut" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +462,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>winsor</t>
+          <t>transform</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -512,7 +513,11 @@
       <c r="H2" t="n">
         <v>7</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>aucune</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>mediane</t>
@@ -520,7 +525,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>porte-a-porte du meilleur mode hors voiture-tout-le-trajet ; le TER inclut le rabattement voiture (park &amp; ride) -&gt; 0 NaN</t>
+          <t>park &amp; ride TER inclus ; 0 NaN</t>
         </is>
       </c>
     </row>
@@ -563,7 +568,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -573,7 +578,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>meilleur trajet alternatif / temps voiture pure ; proche de 1 = le park &amp; ride ne bat pas la voiture -&gt; captif ; 0 NaN</t>
+          <t>meilleur trajet alternatif / temps voiture</t>
         </is>
       </c>
     </row>
@@ -593,17 +598,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>option_sans_voiture</t>
+          <t>part_actifs_tc_pct_2022</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Existe-t-il une option 100% sans voiture ?</t>
+          <t>Part des actifs qui prennent deja le TC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>transport_communes_candidates.csv</t>
+          <t>dynamiques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -612,9 +617,13 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>0</t>
@@ -622,7 +631,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>binaire 0/1 ; 287/411 communes ont un trajet sans voiture du tout</t>
+          <t>RP 2022 (mesure, pas modele) ; valide le pilier (r=0,53 avec le score)</t>
         </is>
       </c>
     </row>
@@ -665,7 +674,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -714,11 +723,11 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -728,7 +737,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>abo TER/Ilevia net du remboursement 50% ; NOTE : pour le park &amp; ride ne compte pas la possession + le rabattement voiture (~+30 EUR/mois)</t>
+          <t>abo TER/Ilevia net du remboursement 50%</t>
         </is>
       </c>
     </row>
@@ -771,7 +780,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -781,7 +790,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>temps pointe / temps fluide (TomTom) ; pese aussi sur le rabattement voiture vers la gare ; fichier bouchons_communes_lille.csv</t>
+          <t>pointe / fluide (TomTom)</t>
         </is>
       </c>
     </row>
@@ -824,7 +833,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -834,7 +843,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>temps routier moyen vers la gare la plus proche (BPE)</t>
+          <t>temps routier moyen (BPE)</t>
         </is>
       </c>
     </row>
@@ -877,7 +886,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>p90</t>
+          <t>log</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,50 +896,50 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>km d'amenagements cyclables utilitaires / 1000 hab (Ecolab/Geovelo 2025)</t>
+          <t>km / 1000 hab (Ecolab/Geovelo 2025)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>prix_immobilier</t>
+          <t>sante</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Prix de l'immobilier</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>prix_maison_m2</t>
+          <t>apl_mg_m65</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Prix des maisons au m2</t>
+          <t>Acces aux medecins generalistes (&lt;= 65 ans)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>immobilier_communes_candidates.csv</t>
+          <t>sante_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>p5_p95</t>
+          <t>aucune</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -940,50 +949,50 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>DVF transactions reelles 2023-2025 (mediane communale) ; winsor DEUX queues : les prix planchers (marche en detresse) ne scorent pas 20/20</t>
+          <t>APL DREES 2024</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>prix_immobilier</t>
+          <t>sante</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prix de l'immobilier</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>loyers_maison_m2</t>
+          <t>apl_dent</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Loyers des maisons au m2</t>
+          <t>Acces aux chirurgiens-dentistes</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>immobilier_communes_candidates.csv</t>
+          <t>sante_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>p5_p95</t>
+          <t>aucune</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -993,37 +1002,37 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Carte des loyers 2025 (indicateur d'annonce predit, CGDD/ANIL)</t>
+          <t>APL DREES 2024 (profession la plus tendue)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>prix_immobilier</t>
+          <t>sante</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prix de l'immobilier</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>loyers_appart_m2</t>
+          <t>acces_urgences_moy_min</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Loyers des appartements au m2</t>
+          <t>Temps d'acces aux urgences</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>immobilier_communes_candidates.csv</t>
+          <t>sante_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1032,11 +1041,11 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>p5_p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1046,7 +1055,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Carte des loyers 2025 ; pertinent surtout pour les communes MEL (locatif)</t>
+          <t>BPE 2025</t>
         </is>
       </c>
     </row>
@@ -1066,12 +1075,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>apl_mg_m65</t>
+          <t>acces_maternite_moy_min</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Acces aux medecins generalistes (&lt;= 65 ans)</t>
+          <t>Temps d'acces a une maternite</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1081,13 +1090,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>7</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>winsor_p95</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>mediane</t>
@@ -1095,19 +1108,19 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>APL DREES 2024, indicateur prospectif</t>
+          <t>BPE 2025</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sante</t>
+          <t>education</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Éducation &amp; petite enfance</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1115,17 +1128,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>apl_dent</t>
+          <t>couverture_petite_enfance_epci</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Acces aux chirurgiens-dentistes</t>
+          <t>Couverture petite enfance</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>sante_communes_candidates.csv</t>
+          <t>education_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1134,9 +1147,13 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>aucune</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>mediane</t>
@@ -1144,19 +1161,19 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>APL DREES 2024 (profession la plus tendue)</t>
+          <t>CNAF 2023, tous modes, niveau EPCI</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sante</t>
+          <t>education</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Éducation &amp; petite enfance</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1164,17 +1181,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>acces_urgences_moy_min</t>
+          <t>acces_college_moy_min</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Temps d'acces aux urgences</t>
+          <t>Temps d'acces a un college</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>sante_communes_candidates.csv</t>
+          <t>education_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1187,7 +1204,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1197,19 +1214,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>BPE 2025, temps routier moyen pondere pop</t>
+          <t>BPE 2025</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sante</t>
+          <t>education</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Éducation &amp; petite enfance</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1217,17 +1234,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>acces_maternite_moy_min</t>
+          <t>acces_lycee_moy_min</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Temps d'acces a une maternite</t>
+          <t>Temps d'acces a un lycee</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>sante_communes_candidates.csv</t>
+          <t>education_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1236,11 +1253,11 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1257,12 +1274,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sante</t>
+          <t>cadre_urbain</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Cadre urbain &amp; logement</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1270,30 +1287,30 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>apl_mg_evol_pct</t>
+          <t>part_logts_vacants</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Trajectoire des generalistes 2022-&gt;2024</t>
+          <t>Part de logements vacants</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>sante_communes_candidates.csv</t>
+          <t>cadre_urbain_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>p5_p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1303,19 +1320,19 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>en baisse dans 296/411 communes ; a lire en tendance</t>
+          <t>INSEE RP 2023 ; proxy vitalite du tissu</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>cadre_urbain</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Éducation &amp; petite enfance</t>
+          <t>Cadre urbain &amp; logement</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1323,28 +1340,32 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>couverture_petite_enfance_epci</t>
+          <t>part_passoires_pct</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Couverture petite enfance</t>
+          <t>Part de passoires thermiques (DPE F-G)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>education_communes_candidates.csv</t>
+          <t>dpe_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>winsor_p95</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
           <t>mediane</t>
@@ -1352,19 +1373,19 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>CNAF 2023, tous modes de garde, niveau EPCI</t>
+          <t>ADEME DPE (echantillon transactions)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Éducation &amp; petite enfance</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1372,17 +1393,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>acces_college_moy_min</t>
+          <t>air_no2_ugm3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Temps d'acces a un college</t>
+          <t>Qualite de l'air : NO2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>education_communes_candidates.csv</t>
+          <t>air_stations_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1391,11 +1412,11 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>aucune</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1405,19 +1426,19 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>BPE 2025</t>
+          <t>concentration annuelle a la station de fond la plus proche (~8 km med) ; indicateur directionnel</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Éducation &amp; petite enfance</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1425,17 +1446,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>acces_lycee_moy_min</t>
+          <t>artif_pct_2009_2024</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Temps d'acces a un lycee</t>
+          <t>Rythme d'artificialisation des sols</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>education_communes_candidates.csv</t>
+          <t>environnement_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1444,11 +1465,11 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1458,19 +1479,19 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>BPE 2025</t>
+          <t>CEREMA 2009-2024</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Éducation &amp; petite enfance</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1478,77 +1499,85 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>college_sur_place</t>
+          <t>imper_pct_2021</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>College dans la commune</t>
+          <t>Impermeabilisation des sols</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>education_communes_candidates.csv</t>
+          <t>environnement_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H21" t="n">
         <v>2</v>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>winsor_p95</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>mediane</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>CEREMA 2021 ; correle densite urbaine</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>commerces</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Commerces &amp; services</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>commerces_essentiels_sur_place</t>
+          <t>catnat_inondation_depuis_2010_n</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Panier de commerces essentiels sur place</t>
+          <t>Inondations recentes</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>commerces_communes_candidates.csv</t>
+          <t>georisques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>winsor_p95</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
           <t>0</t>
@@ -1556,37 +1585,37 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>0-7 : boulangerie, boucherie, epicerie/superette, pharmacie, poste, ecole, medecin</t>
+          <t>arretes CatNat inondation depuis 2010</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>commerces</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Commerces &amp; services</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>acces_supermarche_moy_min</t>
+          <t>rga_pct_moyen_fort</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Temps d'acces a un supermarche</t>
+          <t>Retrait-gonflement des argiles (exposition)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>commerces_communes_candidates.csv</t>
+          <t>rga_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1595,33 +1624,33 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>aucune</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>mediane</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>BPE 2025</t>
+          <t>part surface communale en alea moyen+fort (DREAL/BRGM)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>commerces</t>
+          <t>securite</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Commerces &amp; services</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1629,52 +1658,52 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>resto_pour_1000hab</t>
+          <t>cambriolages_taux</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Restaurants pour 1000 habitants</t>
+          <t>Taux de cambriolages</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>commerces_communes_candidates.csv</t>
+          <t>securite_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>mediane</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>BPE stock 2024, winsorise (artefact zones commerciales)</t>
+          <t>SSMSI moy. 2022-2024 ; ~45% des cellules estimees</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sport_nature</t>
+          <t>securite</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1682,30 +1711,30 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>surf_ev_m2_par_hab</t>
+          <t>degradations_taux</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Espaces verts (m2 par habitant)</t>
+          <t>Taux de degradations volontaires</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>sport_nature_communes_candidates.csv</t>
+          <t>securite_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1715,19 +1744,19 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>parcs/jardins/bois OSM x population</t>
+          <t>SSMSI moy. 2022-2024</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sport_nature</t>
+          <t>commerces</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
+          <t>Commerces &amp; services</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1735,17 +1764,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>clubs_pour_1000hab</t>
+          <t>commerces_essentiels_sur_place</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Clubs sportifs pour 1000 habitants</t>
+          <t>Panier de commerces essentiels sur place</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>sport_nature_communes_candidates.csv</t>
+          <t>commerces_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1758,29 +1787,29 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>aucune</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>mediane</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>INJEP 2023</t>
+          <t>0-7 : boulangerie, boucherie, epicerie, pharmacie, poste, ecole, medecin</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sport_nature</t>
+          <t>commerces</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
+          <t>Commerces &amp; services</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1788,17 +1817,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>acces_piscine_moy_min</t>
+          <t>acces_supermarche_moy_min</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Temps d'acces a une piscine</t>
+          <t>Temps d'acces a un supermarche</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>sport_nature_communes_candidates.csv</t>
+          <t>commerces_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1807,11 +1836,11 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1828,12 +1857,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sport_nature</t>
+          <t>commerces</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
+          <t>Commerces &amp; services</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1841,17 +1870,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>acces_randonnee_moy_min</t>
+          <t>acces_boulangerie_moy_min</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Temps d'acces a un sentier de randonnee</t>
+          <t>Temps d'acces a une boulangerie</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>sport_nature_communes_candidates.csv</t>
+          <t>commerces_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1860,11 +1889,11 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1881,12 +1910,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>securite</t>
+          <t>commerces</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Commerces &amp; services</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1894,52 +1923,52 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>cambriolages_taux</t>
+          <t>resto_pour_1000hab</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Taux de cambriolages</t>
+          <t>Restaurants pour 1000 habitants</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>securite_communes_candidates.csv</t>
+          <t>commerces_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>mediane</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>SSMSI, moyenne 2022-2024, pour 1000 logements ; ~45% des cellules estimees</t>
+          <t>BPE stock 2024 (winsor : artefact zones commerciales)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>securite</t>
+          <t>sport_nature</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Sport &amp; nature</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1947,30 +1976,30 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>degradations_taux</t>
+          <t>surf_ev_m2_par_hab</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Taux de degradations volontaires</t>
+          <t>Espaces verts (m2 par habitant)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>securite_communes_candidates.csv</t>
+          <t>sport_nature_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>log</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1980,19 +2009,19 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>SSMSI moy. 2022-2024</t>
+          <t>parcs/jardins/bois OSM x population</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>securite</t>
+          <t>sport_nature</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Sport &amp; nature</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2000,22 +2029,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>vols_sans_violence_taux</t>
+          <t>clubs_pour_1000hab</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Taux de vols sans violence</t>
+          <t>Clubs sportifs pour 1000 habitants</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>securite_communes_candidates.csv</t>
+          <t>sport_nature_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -2023,7 +2052,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>log</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2033,19 +2062,19 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>SSMSI moy. 2022-2024</t>
+          <t>INJEP 2023</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>securite</t>
+          <t>sport_nature</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Sport &amp; nature</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2053,17 +2082,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>vols_vehicules_taux</t>
+          <t>acces_piscine_moy_min</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Taux de vols lies aux vehicules</t>
+          <t>Temps d'acces a une piscine</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>securite_communes_candidates.csv</t>
+          <t>sport_nature_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2076,7 +2105,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2086,37 +2115,37 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>fusion vols_de_vehicule + vols_dans_vehicules (SSMSI) ; pertinent pour qui se gare a la gare</t>
+          <t>BPE 2025</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>sport_nature</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Sport &amp; nature</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>air_pct_jours_degrades</t>
+          <t>acces_randonnee_moy_min</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Qualite de l'air : jours degrades</t>
+          <t>Temps d'acces a un sentier de randonnee</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>environnement_communes_candidates.csv</t>
+          <t>sport_nature_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2125,9 +2154,13 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
-      </c>
-      <c r="I33" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>winsor_p95</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
           <t>mediane</t>
@@ -2135,50 +2168,50 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>% de jours indice ATMO &gt;= 3 (jan-juil 2026, 169j) ; discrimine tres peu -&gt; poids 1 en attendant les concentrations NO2/PM modelisees (V1.1)</t>
+          <t>BPE 2025</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>dynamique</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Dynamique résidentielle</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>artif_pct_2009_2024</t>
+          <t>taux_var_pop_16_22_pct_an</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Rythme d'artificialisation des sols</t>
+          <t>Croissance de la population 2016-2022</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>environnement_communes_candidates.csv</t>
+          <t>dynamiques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p5_p95</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2188,50 +2221,50 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>CEREMA, flux 2009-2024</t>
+          <t>taux annuel moyen (Insee RP)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>dynamique</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Dynamique résidentielle</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>imper_pct_2021</t>
+          <t>accel_pop_pts</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Impermeabilisation des sols</t>
+          <t>Acceleration demographique</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>environnement_communes_candidates.csv</t>
+          <t>dynamiques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p5_p95</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2241,86 +2274,90 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>CEREMA 2021 ; correle a la densite urbaine (tension editoriale)</t>
+          <t>var. 16-22 moins var. 11-16 (pts)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>dynamique</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Dynamique résidentielle</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>risque_minier</t>
+          <t>arrivants_actifs_pour_1000hab</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Alea minier</t>
+          <t>Arrivee d'actifs (25-54 ans)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>georisques_communes_candidates.csv</t>
+          <t>dynamiques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>inverser</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H36" t="n">
         <v>3</v>
       </c>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>mediane</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>0/1 ; affaissement, effondrement, gaz de mine (113 communes)</t>
+          <t>residaient dans une autre commune 1 an avant (IRAN)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>dynamique</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Dynamique résidentielle</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>catnat_inondation_depuis_2010_n</t>
+          <t>indice_vieillissement_2022</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Inondations recentes</t>
+          <t>Vieillissement de la population</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>georisques_communes_candidates.csv</t>
+          <t>dynamiques_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2333,47 +2370,47 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>mediane</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>nb d'arretes CatNat inondation depuis 2010</t>
+          <t>65+ pour 100 jeunes de -20 ans</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>cout_logement</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Coût du logement</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>rga_pct_moyen_fort</t>
+          <t>prix_maison_m2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Retrait-gonflement des argiles (exposition)</t>
+          <t>Prix des maisons au m2</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>rga_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2382,47 +2419,51 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
-      </c>
-      <c r="I38" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>winsor_p5_p95</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>mediane</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>part de la surface communale en alea moyen+fort (DREAL HdF / BRGM) ; etude de sol obligatoire avant construction depuis la loi ELAN ; 131 communes majoritairement exposees</t>
+          <t>DVF transactions reelles 2023-2025</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cadre_urbain</t>
+          <t>cout_logement</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cadre urbain &amp; logement</t>
+          <t>Coût du logement</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>part_logts_vacants</t>
+          <t>loyers_maison_m2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Part de logements vacants</t>
+          <t>Loyers des maisons au m2</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>cadre_urbain_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2431,11 +2472,11 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p5_p95</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2445,37 +2486,37 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>INSEE RP 2023 ; proxy de vitalite du tissu urbain</t>
+          <t>Carte des loyers 2025 (annonce predite)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cadre_urbain</t>
+          <t>cout_logement</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cadre urbain &amp; logement</t>
+          <t>Coût du logement</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>part_passoires_pct</t>
+          <t>loyers_appart_m2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Part de passoires thermiques (DPE F-G)</t>
+          <t>Loyers des appartements au m2</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dpe_communes_candidates.csv</t>
+          <t>immobilier_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2484,11 +2525,11 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>winsor_p5_p95</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2498,42 +2539,42 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>ADEME DPE 07/2021-08/2026 ; echantillon de transactions, pas le parc complet</t>
+          <t>Carte des loyers 2025</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cadre_urbain</t>
+          <t>cout_logement</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cadre urbain &amp; logement</t>
+          <t>Coût du logement</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>evol_pop_2016_2022_pct</t>
+          <t>taux_taxe_fonciere_bati</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Dynamique demographique 2016-2022</t>
+          <t>Taux de taxe fonciere</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>cadre_urbain_communes_candidates.csv</t>
+          <t>fiscalite_communes_candidates.csv</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>inverser</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2541,7 +2582,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>p5_p95</t>
+          <t>winsor_p95</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2551,7 +2592,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>INSEE</t>
+          <t>DGFiP 2025, taux global sur le bati</t>
         </is>
       </c>
     </row>
@@ -2566,173 +2607,246 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>theme_libelle</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>n_criteres</t>
+          <t>colonne</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>poids_total</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>etoiles</t>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fichier_source</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>libelle</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cadre urbain &amp; logement</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="n">
-        <v>11</v>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>desserte_directe_faible</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>truthy</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>-0.3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>transport_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>gare de rabattement mal desservie</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Commerces &amp; services</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="n">
-        <v>12</v>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>option_sans_voiture</t>
+        </is>
+      </c>
+      <c r="C3">
+        <f>= 0</f>
+        <v/>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>-0.4</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>transport_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>aucun trajet 100% sans voiture possible</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" t="n">
-        <v>15</v>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>gare_sur_territoire</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>truthy</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>0.2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>transport_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>une gare TER dans la commune</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Prix de l'immobilier</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" t="n">
-        <v>11</v>
+          <t>sante</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>msp_sur_place</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>truthy</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0.2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sante_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>maison de sante pluriprofessionnelle sur place</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Santé</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>21</v>
+          <t>sante</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>acces_urgences_moy_min</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>&gt; 20</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>-0.3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sante_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>urgences a plus de 20 min</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" t="n">
-        <v>15</v>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>college_sur_place</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>= 1</f>
+        <v/>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>0.25</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>education_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>un college dans la commune</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sécurité</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C8" t="n">
-        <v>16</v>
+          <t>environnement</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>risque_minier</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>= 1</f>
+        <v/>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Transport vers Lille</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="n">
-        <v>33</v>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Éducation &amp; petite enfance</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" t="n">
-        <v>17</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
+        <v>-0.3</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>georisques_communes_candidates.csv</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>alea minier (affaissement, gaz de mine)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2746,29 +2860,225 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>theme_libelle</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>libelle</t>
+          <t>n_criteres</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>etoiles_defaut</t>
+          <t>poids_total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>etoiles</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Cadre urbain &amp; logement</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Commerces &amp; services</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Coût du logement</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dynamique résidentielle</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Environnement &amp; risques</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Santé</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sport &amp; nature</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Transport vers Lille</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Éducation &amp; petite enfance</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>theme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>libelle</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>etoiles_defaut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>transport</t>
         </is>
       </c>
@@ -2784,27 +3094,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>prix_immobilier</t>
+          <t>sante</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prix de l'immobilier</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sante</t>
+          <t>education</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Éducation &amp; petite enfance</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2814,12 +3124,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>cadre_urbain</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Éducation &amp; petite enfance</t>
+          <t>Cadre urbain &amp; logement</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2829,57 +3139,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>securite</t>
+          <t>environnement</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Environnement &amp; risques</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cadre_urbain</t>
+          <t>securite</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cadre urbain &amp; logement</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>environnement</t>
+          <t>commerces</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Environnement &amp; risques</t>
+          <t>Commerces &amp; services</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>commerces</t>
+          <t>sport_nature</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Commerces &amp; services</t>
+          <t>Sport &amp; nature</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -2889,16 +3199,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sport_nature</t>
+          <t>dynamique</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sport &amp; nature</t>
+          <t>Dynamique résidentielle</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cout_logement</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Coût du logement</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>